<commit_message>
Booking group,exp del date from carrier feed,re-submission version preserve,modify FC on mapping
</commit_message>
<xml_diff>
--- a/samples/SupplierInput_template.xlsx
+++ b/samples/SupplierInput_template.xlsx
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="67">
   <si>
     <t>Carton_Type</t>
   </si>
@@ -235,9 +235,6 @@
   </si>
   <si>
     <t>Hazardous</t>
-  </si>
-  <si>
-    <t>Expected_Delivery_Date</t>
   </si>
   <si>
     <t>Remarks</t>
@@ -263,7 +260,7 @@
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -290,8 +287,12 @@
       <color rgb="FF1A5276"/>
       <sz val="10"/>
     </font>
+    <font>
+      <color rgb="FF7B3F00"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -333,6 +334,11 @@
         <fgColor rgb="FFD6E8F8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF3CD"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -355,7 +361,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -394,6 +400,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyProtection="1"/>
     <xf numFmtId="164" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1095,8 +1102,7 @@
     <col min="31" max="31" width="18" customWidth="1"/>
     <col min="32" max="32" width="24" customWidth="1"/>
     <col min="33" max="33" width="20" customWidth="1"/>
-    <col min="34" max="34" width="24" customWidth="1"/>
-    <col min="35" max="35" width="30" customWidth="1"/>
+    <col min="34" max="34" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
@@ -1155,7 +1161,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" ht="36" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" ht="36" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>30</v>
       </c>
@@ -1258,16 +1264,13 @@
       <c r="AH3" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="AI3" s="9" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="4" spans="4:34" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E4" s="12"/>
       <c r="F4" s="13"/>
       <c r="G4" s="13"/>
       <c r="I4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="V4" t="s">
         <v>5</v>
@@ -1294,22 +1297,24 @@
         <f>IFERROR((W4*X4*Y4/1000000)*D4,0)</f>
       </c>
       <c r="AD4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG4" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH4" s="13"/>
-    </row>
-    <row r="5" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E5" s="12"/>
       <c r="F5" s="13"/>
       <c r="G5" s="13"/>
       <c r="I5" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P5" s="16">
+        <f>IF($A5="","",IFERROR(INDEX($P$4:P4,MATCH($A5,$A$4:$A4,0)),""))</f>
       </c>
       <c r="V5" t="s">
         <v>5</v>
@@ -1336,22 +1341,24 @@
         <f>IFERROR((W5*X5*Y5/1000000)*D5,0)</f>
       </c>
       <c r="AD5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG5" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH5" s="13"/>
-    </row>
-    <row r="6" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E6" s="12"/>
       <c r="F6" s="13"/>
       <c r="G6" s="13"/>
       <c r="I6" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P6" s="16">
+        <f>IF($A6="","",IFERROR(INDEX($P$4:P5,MATCH($A6,$A$4:$A5,0)),""))</f>
       </c>
       <c r="V6" t="s">
         <v>5</v>
@@ -1378,22 +1385,24 @@
         <f>IFERROR((W6*X6*Y6/1000000)*D6,0)</f>
       </c>
       <c r="AD6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG6" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH6" s="13"/>
-    </row>
-    <row r="7" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E7" s="12"/>
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
       <c r="I7" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P7" s="16">
+        <f>IF($A7="","",IFERROR(INDEX($P$4:P6,MATCH($A7,$A$4:$A6,0)),""))</f>
       </c>
       <c r="V7" t="s">
         <v>5</v>
@@ -1420,22 +1429,24 @@
         <f>IFERROR((W7*X7*Y7/1000000)*D7,0)</f>
       </c>
       <c r="AD7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG7" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH7" s="13"/>
-    </row>
-    <row r="8" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E8" s="12"/>
       <c r="F8" s="13"/>
       <c r="G8" s="13"/>
       <c r="I8" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P8" s="16">
+        <f>IF($A8="","",IFERROR(INDEX($P$4:P7,MATCH($A8,$A$4:$A7,0)),""))</f>
       </c>
       <c r="V8" t="s">
         <v>5</v>
@@ -1462,22 +1473,24 @@
         <f>IFERROR((W8*X8*Y8/1000000)*D8,0)</f>
       </c>
       <c r="AD8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG8" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH8" s="13"/>
-    </row>
-    <row r="9" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="9" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E9" s="12"/>
       <c r="F9" s="13"/>
       <c r="G9" s="13"/>
       <c r="I9" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P9" s="16">
+        <f>IF($A9="","",IFERROR(INDEX($P$4:P8,MATCH($A9,$A$4:$A8,0)),""))</f>
       </c>
       <c r="V9" t="s">
         <v>5</v>
@@ -1504,22 +1517,24 @@
         <f>IFERROR((W9*X9*Y9/1000000)*D9,0)</f>
       </c>
       <c r="AD9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG9" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH9" s="13"/>
-    </row>
-    <row r="10" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E10" s="12"/>
       <c r="F10" s="13"/>
       <c r="G10" s="13"/>
       <c r="I10" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P10" s="16">
+        <f>IF($A10="","",IFERROR(INDEX($P$4:P9,MATCH($A10,$A$4:$A9,0)),""))</f>
       </c>
       <c r="V10" t="s">
         <v>5</v>
@@ -1546,22 +1561,24 @@
         <f>IFERROR((W10*X10*Y10/1000000)*D10,0)</f>
       </c>
       <c r="AD10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG10" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH10" s="13"/>
-    </row>
-    <row r="11" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E11" s="12"/>
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
       <c r="I11" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P11" s="16">
+        <f>IF($A11="","",IFERROR(INDEX($P$4:P10,MATCH($A11,$A$4:$A10,0)),""))</f>
       </c>
       <c r="V11" t="s">
         <v>5</v>
@@ -1588,22 +1605,24 @@
         <f>IFERROR((W11*X11*Y11/1000000)*D11,0)</f>
       </c>
       <c r="AD11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH11" s="13"/>
-    </row>
-    <row r="12" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E12" s="12"/>
       <c r="F12" s="13"/>
       <c r="G12" s="13"/>
       <c r="I12" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P12" s="16">
+        <f>IF($A12="","",IFERROR(INDEX($P$4:P11,MATCH($A12,$A$4:$A11,0)),""))</f>
       </c>
       <c r="V12" t="s">
         <v>5</v>
@@ -1630,22 +1649,24 @@
         <f>IFERROR((W12*X12*Y12/1000000)*D12,0)</f>
       </c>
       <c r="AD12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG12" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH12" s="13"/>
-    </row>
-    <row r="13" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E13" s="12"/>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
       <c r="I13" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P13" s="16">
+        <f>IF($A13="","",IFERROR(INDEX($P$4:P12,MATCH($A13,$A$4:$A12,0)),""))</f>
       </c>
       <c r="V13" t="s">
         <v>5</v>
@@ -1672,22 +1693,24 @@
         <f>IFERROR((W13*X13*Y13/1000000)*D13,0)</f>
       </c>
       <c r="AD13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG13" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH13" s="13"/>
-    </row>
-    <row r="14" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="14" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E14" s="12"/>
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
       <c r="I14" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P14" s="16">
+        <f>IF($A14="","",IFERROR(INDEX($P$4:P13,MATCH($A14,$A$4:$A13,0)),""))</f>
       </c>
       <c r="V14" t="s">
         <v>5</v>
@@ -1714,22 +1737,24 @@
         <f>IFERROR((W14*X14*Y14/1000000)*D14,0)</f>
       </c>
       <c r="AD14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG14" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH14" s="13"/>
-    </row>
-    <row r="15" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="15" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E15" s="12"/>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
       <c r="I15" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P15" s="16">
+        <f>IF($A15="","",IFERROR(INDEX($P$4:P14,MATCH($A15,$A$4:$A14,0)),""))</f>
       </c>
       <c r="V15" t="s">
         <v>5</v>
@@ -1756,22 +1781,24 @@
         <f>IFERROR((W15*X15*Y15/1000000)*D15,0)</f>
       </c>
       <c r="AD15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG15" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH15" s="13"/>
-    </row>
-    <row r="16" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E16" s="12"/>
       <c r="F16" s="13"/>
       <c r="G16" s="13"/>
       <c r="I16" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P16" s="16">
+        <f>IF($A16="","",IFERROR(INDEX($P$4:P15,MATCH($A16,$A$4:$A15,0)),""))</f>
       </c>
       <c r="V16" t="s">
         <v>5</v>
@@ -1798,22 +1825,24 @@
         <f>IFERROR((W16*X16*Y16/1000000)*D16,0)</f>
       </c>
       <c r="AD16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG16" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH16" s="13"/>
-    </row>
-    <row r="17" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="17" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E17" s="12"/>
       <c r="F17" s="13"/>
       <c r="G17" s="13"/>
       <c r="I17" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P17" s="16">
+        <f>IF($A17="","",IFERROR(INDEX($P$4:P16,MATCH($A17,$A$4:$A16,0)),""))</f>
       </c>
       <c r="V17" t="s">
         <v>5</v>
@@ -1840,22 +1869,24 @@
         <f>IFERROR((W17*X17*Y17/1000000)*D17,0)</f>
       </c>
       <c r="AD17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG17" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH17" s="13"/>
-    </row>
-    <row r="18" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="18" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E18" s="12"/>
       <c r="F18" s="13"/>
       <c r="G18" s="13"/>
       <c r="I18" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P18" s="16">
+        <f>IF($A18="","",IFERROR(INDEX($P$4:P17,MATCH($A18,$A$4:$A17,0)),""))</f>
       </c>
       <c r="V18" t="s">
         <v>5</v>
@@ -1882,22 +1913,24 @@
         <f>IFERROR((W18*X18*Y18/1000000)*D18,0)</f>
       </c>
       <c r="AD18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE18" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG18" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH18" s="13"/>
-    </row>
-    <row r="19" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="19" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E19" s="12"/>
       <c r="F19" s="13"/>
       <c r="G19" s="13"/>
       <c r="I19" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P19" s="16">
+        <f>IF($A19="","",IFERROR(INDEX($P$4:P18,MATCH($A19,$A$4:$A18,0)),""))</f>
       </c>
       <c r="V19" t="s">
         <v>5</v>
@@ -1924,22 +1957,24 @@
         <f>IFERROR((W19*X19*Y19/1000000)*D19,0)</f>
       </c>
       <c r="AD19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE19" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG19" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH19" s="13"/>
-    </row>
-    <row r="20" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E20" s="12"/>
       <c r="F20" s="13"/>
       <c r="G20" s="13"/>
       <c r="I20" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P20" s="16">
+        <f>IF($A20="","",IFERROR(INDEX($P$4:P19,MATCH($A20,$A$4:$A19,0)),""))</f>
       </c>
       <c r="V20" t="s">
         <v>5</v>
@@ -1966,22 +2001,24 @@
         <f>IFERROR((W20*X20*Y20/1000000)*D20,0)</f>
       </c>
       <c r="AD20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG20" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH20" s="13"/>
-    </row>
-    <row r="21" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="21" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E21" s="12"/>
       <c r="F21" s="13"/>
       <c r="G21" s="13"/>
       <c r="I21" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P21" s="16">
+        <f>IF($A21="","",IFERROR(INDEX($P$4:P20,MATCH($A21,$A$4:$A20,0)),""))</f>
       </c>
       <c r="V21" t="s">
         <v>5</v>
@@ -2008,22 +2045,24 @@
         <f>IFERROR((W21*X21*Y21/1000000)*D21,0)</f>
       </c>
       <c r="AD21" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE21" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG21" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH21" s="13"/>
-    </row>
-    <row r="22" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="22" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E22" s="12"/>
       <c r="F22" s="13"/>
       <c r="G22" s="13"/>
       <c r="I22" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P22" s="16">
+        <f>IF($A22="","",IFERROR(INDEX($P$4:P21,MATCH($A22,$A$4:$A21,0)),""))</f>
       </c>
       <c r="V22" t="s">
         <v>5</v>
@@ -2050,22 +2089,24 @@
         <f>IFERROR((W22*X22*Y22/1000000)*D22,0)</f>
       </c>
       <c r="AD22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH22" s="13"/>
-    </row>
-    <row r="23" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="23" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E23" s="12"/>
       <c r="F23" s="13"/>
       <c r="G23" s="13"/>
       <c r="I23" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P23" s="16">
+        <f>IF($A23="","",IFERROR(INDEX($P$4:P22,MATCH($A23,$A$4:$A22,0)),""))</f>
       </c>
       <c r="V23" t="s">
         <v>5</v>
@@ -2092,22 +2133,24 @@
         <f>IFERROR((W23*X23*Y23/1000000)*D23,0)</f>
       </c>
       <c r="AD23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE23" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG23" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH23" s="13"/>
-    </row>
-    <row r="24" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="24" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E24" s="12"/>
       <c r="F24" s="13"/>
       <c r="G24" s="13"/>
       <c r="I24" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P24" s="16">
+        <f>IF($A24="","",IFERROR(INDEX($P$4:P23,MATCH($A24,$A$4:$A23,0)),""))</f>
       </c>
       <c r="V24" t="s">
         <v>5</v>
@@ -2134,22 +2177,24 @@
         <f>IFERROR((W24*X24*Y24/1000000)*D24,0)</f>
       </c>
       <c r="AD24" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE24" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG24" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH24" s="13"/>
-    </row>
-    <row r="25" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="25" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E25" s="12"/>
       <c r="F25" s="13"/>
       <c r="G25" s="13"/>
       <c r="I25" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P25" s="16">
+        <f>IF($A25="","",IFERROR(INDEX($P$4:P24,MATCH($A25,$A$4:$A24,0)),""))</f>
       </c>
       <c r="V25" t="s">
         <v>5</v>
@@ -2176,22 +2221,24 @@
         <f>IFERROR((W25*X25*Y25/1000000)*D25,0)</f>
       </c>
       <c r="AD25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE25" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH25" s="13"/>
-    </row>
-    <row r="26" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="26" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E26" s="12"/>
       <c r="F26" s="13"/>
       <c r="G26" s="13"/>
       <c r="I26" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P26" s="16">
+        <f>IF($A26="","",IFERROR(INDEX($P$4:P25,MATCH($A26,$A$4:$A25,0)),""))</f>
       </c>
       <c r="V26" t="s">
         <v>5</v>
@@ -2218,22 +2265,24 @@
         <f>IFERROR((W26*X26*Y26/1000000)*D26,0)</f>
       </c>
       <c r="AD26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE26" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG26" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH26" s="13"/>
-    </row>
-    <row r="27" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="27" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E27" s="12"/>
       <c r="F27" s="13"/>
       <c r="G27" s="13"/>
       <c r="I27" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P27" s="16">
+        <f>IF($A27="","",IFERROR(INDEX($P$4:P26,MATCH($A27,$A$4:$A26,0)),""))</f>
       </c>
       <c r="V27" t="s">
         <v>5</v>
@@ -2260,22 +2309,24 @@
         <f>IFERROR((W27*X27*Y27/1000000)*D27,0)</f>
       </c>
       <c r="AD27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE27" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG27" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH27" s="13"/>
-    </row>
-    <row r="28" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="28" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E28" s="12"/>
       <c r="F28" s="13"/>
       <c r="G28" s="13"/>
       <c r="I28" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P28" s="16">
+        <f>IF($A28="","",IFERROR(INDEX($P$4:P27,MATCH($A28,$A$4:$A27,0)),""))</f>
       </c>
       <c r="V28" t="s">
         <v>5</v>
@@ -2302,22 +2353,24 @@
         <f>IFERROR((W28*X28*Y28/1000000)*D28,0)</f>
       </c>
       <c r="AD28" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE28" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG28" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH28" s="13"/>
-    </row>
-    <row r="29" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="29" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E29" s="12"/>
       <c r="F29" s="13"/>
       <c r="G29" s="13"/>
       <c r="I29" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P29" s="16">
+        <f>IF($A29="","",IFERROR(INDEX($P$4:P28,MATCH($A29,$A$4:$A28,0)),""))</f>
       </c>
       <c r="V29" t="s">
         <v>5</v>
@@ -2344,22 +2397,24 @@
         <f>IFERROR((W29*X29*Y29/1000000)*D29,0)</f>
       </c>
       <c r="AD29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE29" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH29" s="13"/>
-    </row>
-    <row r="30" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="30" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E30" s="12"/>
       <c r="F30" s="13"/>
       <c r="G30" s="13"/>
       <c r="I30" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P30" s="16">
+        <f>IF($A30="","",IFERROR(INDEX($P$4:P29,MATCH($A30,$A$4:$A29,0)),""))</f>
       </c>
       <c r="V30" t="s">
         <v>5</v>
@@ -2386,22 +2441,24 @@
         <f>IFERROR((W30*X30*Y30/1000000)*D30,0)</f>
       </c>
       <c r="AD30" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE30" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG30" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH30" s="13"/>
-    </row>
-    <row r="31" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="31" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E31" s="12"/>
       <c r="F31" s="13"/>
       <c r="G31" s="13"/>
       <c r="I31" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P31" s="16">
+        <f>IF($A31="","",IFERROR(INDEX($P$4:P30,MATCH($A31,$A$4:$A30,0)),""))</f>
       </c>
       <c r="V31" t="s">
         <v>5</v>
@@ -2428,22 +2485,24 @@
         <f>IFERROR((W31*X31*Y31/1000000)*D31,0)</f>
       </c>
       <c r="AD31" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE31" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG31" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH31" s="13"/>
-    </row>
-    <row r="32" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="32" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E32" s="12"/>
       <c r="F32" s="13"/>
       <c r="G32" s="13"/>
       <c r="I32" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P32" s="16">
+        <f>IF($A32="","",IFERROR(INDEX($P$4:P31,MATCH($A32,$A$4:$A31,0)),""))</f>
       </c>
       <c r="V32" t="s">
         <v>5</v>
@@ -2470,22 +2529,24 @@
         <f>IFERROR((W32*X32*Y32/1000000)*D32,0)</f>
       </c>
       <c r="AD32" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE32" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG32" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH32" s="13"/>
-    </row>
-    <row r="33" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="33" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E33" s="12"/>
       <c r="F33" s="13"/>
       <c r="G33" s="13"/>
       <c r="I33" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P33" s="16">
+        <f>IF($A33="","",IFERROR(INDEX($P$4:P32,MATCH($A33,$A$4:$A32,0)),""))</f>
       </c>
       <c r="V33" t="s">
         <v>5</v>
@@ -2512,22 +2573,24 @@
         <f>IFERROR((W33*X33*Y33/1000000)*D33,0)</f>
       </c>
       <c r="AD33" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE33" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG33" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH33" s="13"/>
-    </row>
-    <row r="34" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="34" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E34" s="12"/>
       <c r="F34" s="13"/>
       <c r="G34" s="13"/>
       <c r="I34" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P34" s="16">
+        <f>IF($A34="","",IFERROR(INDEX($P$4:P33,MATCH($A34,$A$4:$A33,0)),""))</f>
       </c>
       <c r="V34" t="s">
         <v>5</v>
@@ -2554,22 +2617,24 @@
         <f>IFERROR((W34*X34*Y34/1000000)*D34,0)</f>
       </c>
       <c r="AD34" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE34" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG34" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH34" s="13"/>
-    </row>
-    <row r="35" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="35" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E35" s="12"/>
       <c r="F35" s="13"/>
       <c r="G35" s="13"/>
       <c r="I35" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P35" s="16">
+        <f>IF($A35="","",IFERROR(INDEX($P$4:P34,MATCH($A35,$A$4:$A34,0)),""))</f>
       </c>
       <c r="V35" t="s">
         <v>5</v>
@@ -2596,22 +2661,24 @@
         <f>IFERROR((W35*X35*Y35/1000000)*D35,0)</f>
       </c>
       <c r="AD35" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE35" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG35" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH35" s="13"/>
-    </row>
-    <row r="36" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="36" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E36" s="12"/>
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
       <c r="I36" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P36" s="16">
+        <f>IF($A36="","",IFERROR(INDEX($P$4:P35,MATCH($A36,$A$4:$A35,0)),""))</f>
       </c>
       <c r="V36" t="s">
         <v>5</v>
@@ -2638,22 +2705,24 @@
         <f>IFERROR((W36*X36*Y36/1000000)*D36,0)</f>
       </c>
       <c r="AD36" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE36" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG36" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH36" s="13"/>
-    </row>
-    <row r="37" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="37" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E37" s="12"/>
       <c r="F37" s="13"/>
       <c r="G37" s="13"/>
       <c r="I37" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P37" s="16">
+        <f>IF($A37="","",IFERROR(INDEX($P$4:P36,MATCH($A37,$A$4:$A36,0)),""))</f>
       </c>
       <c r="V37" t="s">
         <v>5</v>
@@ -2680,22 +2749,24 @@
         <f>IFERROR((W37*X37*Y37/1000000)*D37,0)</f>
       </c>
       <c r="AD37" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE37" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG37" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH37" s="13"/>
-    </row>
-    <row r="38" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="38" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E38" s="12"/>
       <c r="F38" s="13"/>
       <c r="G38" s="13"/>
       <c r="I38" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P38" s="16">
+        <f>IF($A38="","",IFERROR(INDEX($P$4:P37,MATCH($A38,$A$4:$A37,0)),""))</f>
       </c>
       <c r="V38" t="s">
         <v>5</v>
@@ -2722,22 +2793,24 @@
         <f>IFERROR((W38*X38*Y38/1000000)*D38,0)</f>
       </c>
       <c r="AD38" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE38" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG38" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH38" s="13"/>
-    </row>
-    <row r="39" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="39" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E39" s="12"/>
       <c r="F39" s="13"/>
       <c r="G39" s="13"/>
       <c r="I39" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P39" s="16">
+        <f>IF($A39="","",IFERROR(INDEX($P$4:P38,MATCH($A39,$A$4:$A38,0)),""))</f>
       </c>
       <c r="V39" t="s">
         <v>5</v>
@@ -2764,22 +2837,24 @@
         <f>IFERROR((W39*X39*Y39/1000000)*D39,0)</f>
       </c>
       <c r="AD39" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE39" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG39" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH39" s="13"/>
-    </row>
-    <row r="40" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="40" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E40" s="12"/>
       <c r="F40" s="13"/>
       <c r="G40" s="13"/>
       <c r="I40" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P40" s="16">
+        <f>IF($A40="","",IFERROR(INDEX($P$4:P39,MATCH($A40,$A$4:$A39,0)),""))</f>
       </c>
       <c r="V40" t="s">
         <v>5</v>
@@ -2806,22 +2881,24 @@
         <f>IFERROR((W40*X40*Y40/1000000)*D40,0)</f>
       </c>
       <c r="AD40" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE40" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG40" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH40" s="13"/>
-    </row>
-    <row r="41" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="41" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E41" s="12"/>
       <c r="F41" s="13"/>
       <c r="G41" s="13"/>
       <c r="I41" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P41" s="16">
+        <f>IF($A41="","",IFERROR(INDEX($P$4:P40,MATCH($A41,$A$4:$A40,0)),""))</f>
       </c>
       <c r="V41" t="s">
         <v>5</v>
@@ -2848,22 +2925,24 @@
         <f>IFERROR((W41*X41*Y41/1000000)*D41,0)</f>
       </c>
       <c r="AD41" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE41" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG41" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH41" s="13"/>
-    </row>
-    <row r="42" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="42" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E42" s="12"/>
       <c r="F42" s="13"/>
       <c r="G42" s="13"/>
       <c r="I42" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P42" s="16">
+        <f>IF($A42="","",IFERROR(INDEX($P$4:P41,MATCH($A42,$A$4:$A41,0)),""))</f>
       </c>
       <c r="V42" t="s">
         <v>5</v>
@@ -2890,22 +2969,24 @@
         <f>IFERROR((W42*X42*Y42/1000000)*D42,0)</f>
       </c>
       <c r="AD42" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE42" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG42" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH42" s="13"/>
-    </row>
-    <row r="43" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="43" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E43" s="12"/>
       <c r="F43" s="13"/>
       <c r="G43" s="13"/>
       <c r="I43" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P43" s="16">
+        <f>IF($A43="","",IFERROR(INDEX($P$4:P42,MATCH($A43,$A$4:$A42,0)),""))</f>
       </c>
       <c r="V43" t="s">
         <v>5</v>
@@ -2932,22 +3013,24 @@
         <f>IFERROR((W43*X43*Y43/1000000)*D43,0)</f>
       </c>
       <c r="AD43" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE43" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG43" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH43" s="13"/>
-    </row>
-    <row r="44" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="44" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E44" s="12"/>
       <c r="F44" s="13"/>
       <c r="G44" s="13"/>
       <c r="I44" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P44" s="16">
+        <f>IF($A44="","",IFERROR(INDEX($P$4:P43,MATCH($A44,$A$4:$A43,0)),""))</f>
       </c>
       <c r="V44" t="s">
         <v>5</v>
@@ -2974,22 +3057,24 @@
         <f>IFERROR((W44*X44*Y44/1000000)*D44,0)</f>
       </c>
       <c r="AD44" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE44" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG44" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH44" s="13"/>
-    </row>
-    <row r="45" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="45" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E45" s="12"/>
       <c r="F45" s="13"/>
       <c r="G45" s="13"/>
       <c r="I45" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P45" s="16">
+        <f>IF($A45="","",IFERROR(INDEX($P$4:P44,MATCH($A45,$A$4:$A44,0)),""))</f>
       </c>
       <c r="V45" t="s">
         <v>5</v>
@@ -3016,22 +3101,24 @@
         <f>IFERROR((W45*X45*Y45/1000000)*D45,0)</f>
       </c>
       <c r="AD45" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE45" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG45" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH45" s="13"/>
-    </row>
-    <row r="46" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="46" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E46" s="12"/>
       <c r="F46" s="13"/>
       <c r="G46" s="13"/>
       <c r="I46" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P46" s="16">
+        <f>IF($A46="","",IFERROR(INDEX($P$4:P45,MATCH($A46,$A$4:$A45,0)),""))</f>
       </c>
       <c r="V46" t="s">
         <v>5</v>
@@ -3058,22 +3145,24 @@
         <f>IFERROR((W46*X46*Y46/1000000)*D46,0)</f>
       </c>
       <c r="AD46" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE46" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG46" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH46" s="13"/>
-    </row>
-    <row r="47" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="47" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E47" s="12"/>
       <c r="F47" s="13"/>
       <c r="G47" s="13"/>
       <c r="I47" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P47" s="16">
+        <f>IF($A47="","",IFERROR(INDEX($P$4:P46,MATCH($A47,$A$4:$A46,0)),""))</f>
       </c>
       <c r="V47" t="s">
         <v>5</v>
@@ -3100,22 +3189,24 @@
         <f>IFERROR((W47*X47*Y47/1000000)*D47,0)</f>
       </c>
       <c r="AD47" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE47" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG47" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH47" s="13"/>
-    </row>
-    <row r="48" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="48" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E48" s="12"/>
       <c r="F48" s="13"/>
       <c r="G48" s="13"/>
       <c r="I48" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P48" s="16">
+        <f>IF($A48="","",IFERROR(INDEX($P$4:P47,MATCH($A48,$A$4:$A47,0)),""))</f>
       </c>
       <c r="V48" t="s">
         <v>5</v>
@@ -3142,22 +3233,24 @@
         <f>IFERROR((W48*X48*Y48/1000000)*D48,0)</f>
       </c>
       <c r="AD48" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE48" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG48" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH48" s="13"/>
-    </row>
-    <row r="49" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="49" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E49" s="12"/>
       <c r="F49" s="13"/>
       <c r="G49" s="13"/>
       <c r="I49" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P49" s="16">
+        <f>IF($A49="","",IFERROR(INDEX($P$4:P48,MATCH($A49,$A$4:$A48,0)),""))</f>
       </c>
       <c r="V49" t="s">
         <v>5</v>
@@ -3184,22 +3277,24 @@
         <f>IFERROR((W49*X49*Y49/1000000)*D49,0)</f>
       </c>
       <c r="AD49" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG49" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH49" s="13"/>
-    </row>
-    <row r="50" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="50" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E50" s="12"/>
       <c r="F50" s="13"/>
       <c r="G50" s="13"/>
       <c r="I50" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P50" s="16">
+        <f>IF($A50="","",IFERROR(INDEX($P$4:P49,MATCH($A50,$A$4:$A49,0)),""))</f>
       </c>
       <c r="V50" t="s">
         <v>5</v>
@@ -3226,22 +3321,24 @@
         <f>IFERROR((W50*X50*Y50/1000000)*D50,0)</f>
       </c>
       <c r="AD50" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE50" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG50" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH50" s="13"/>
-    </row>
-    <row r="51" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="51" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E51" s="12"/>
       <c r="F51" s="13"/>
       <c r="G51" s="13"/>
       <c r="I51" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P51" s="16">
+        <f>IF($A51="","",IFERROR(INDEX($P$4:P50,MATCH($A51,$A$4:$A50,0)),""))</f>
       </c>
       <c r="V51" t="s">
         <v>5</v>
@@ -3268,22 +3365,24 @@
         <f>IFERROR((W51*X51*Y51/1000000)*D51,0)</f>
       </c>
       <c r="AD51" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE51" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG51" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH51" s="13"/>
-    </row>
-    <row r="52" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="52" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E52" s="12"/>
       <c r="F52" s="13"/>
       <c r="G52" s="13"/>
       <c r="I52" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P52" s="16">
+        <f>IF($A52="","",IFERROR(INDEX($P$4:P51,MATCH($A52,$A$4:$A51,0)),""))</f>
       </c>
       <c r="V52" t="s">
         <v>5</v>
@@ -3310,22 +3409,24 @@
         <f>IFERROR((W52*X52*Y52/1000000)*D52,0)</f>
       </c>
       <c r="AD52" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE52" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG52" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH52" s="13"/>
-    </row>
-    <row r="53" spans="4:34" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="53" spans="4:33" x14ac:dyDescent="0.25">
       <c r="E53" s="12"/>
       <c r="F53" s="13"/>
       <c r="G53" s="13"/>
       <c r="I53" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="P53" s="16">
+        <f>IF($A53="","",IFERROR(INDEX($P$4:P52,MATCH($A53,$A$4:$A52,0)),""))</f>
       </c>
       <c r="V53" t="s">
         <v>5</v>
@@ -3352,21 +3453,20 @@
         <f>IFERROR((W53*X53*Y53/1000000)*D53,0)</f>
       </c>
       <c r="AD53" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE53" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG53" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH53" s="13"/>
+        <v>66</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:AI1"/>
   </mergeCells>
-  <dataValidations count="22">
+  <dataValidations count="20">
     <dataValidation type="list" sqref="AD10:AD53">
       <formula1>"Flat,Bulk Flat,Hanging"</formula1>
     </dataValidation>
@@ -3384,12 +3484,6 @@
     </dataValidation>
     <dataValidation type="list" sqref="AG4:AG53">
       <formula1>"Flammable,Glass - Hazardous,Hazardous,N/A"</formula1>
-    </dataValidation>
-    <dataValidation type="date" operator="greaterThan" showErrorMessage="1" errorTitle="Invalid date" error="Enter a valid date (DD/MM/YYYY format)" sqref="AH10:AH53">
-      <formula1>43831</formula1>
-    </dataValidation>
-    <dataValidation type="date" operator="greaterThan" showErrorMessage="1" errorTitle="Invalid date" error="Enter a valid date (DD/MM/YYYY format)" sqref="AH4:AH53">
-      <formula1>43831</formula1>
     </dataValidation>
     <dataValidation type="whole" operator="greaterThan" showErrorMessage="1" errorTitle="Invalid" error="Enter a whole number greater than 0" sqref="D10:D53">
       <formula1>0</formula1>

</xml_diff>